<commit_message>
Preserve tender types and reject data beyond approved columns
</commit_message>
<xml_diff>
--- a/tests-dotnet/fixtures/etp-sample/R001_AdvanceOrder_Collection.xlsx
+++ b/tests-dotnet/fixtures/etp-sample/R001_AdvanceOrder_Collection.xlsx
@@ -771,10 +771,8 @@
       <c r="AF2" t="n">
         <v>0</v>
       </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>SAMPLE</t>
-        </is>
+      <c r="AG2" t="n">
+        <v>19.75</v>
       </c>
       <c r="AH2" t="n">
         <v>0</v>

</xml_diff>